<commit_message>
feat: add interactive UI animations, billing discount segment, selling price rename, and MedEx auto-fill for stock-in
- Enhanced UI with micro-animations, card hover effects, audio feedback, page transitions, and checkout confetti
- Renamed 'last price' to 'Selling Price' across all UI components, APIs, and reports
- Added percentage discount segment in POS billing with real-time recalculations and receipt breakdown
- Implemented MedEx brand detail fetching to auto-fill group category, wholesale trade cost (~88% MRP), and selling price during stock-in
- Resolved ESLint rules and optimized database cache
</commit_message>
<xml_diff>
--- a/reports/report_2026-08-31.xlsx
+++ b/reports/report_2026-08-31.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="75">
   <si>
     <t>Invoice No</t>
   </si>
@@ -221,6 +221,9 @@
   </si>
   <si>
     <t>bottle</t>
+  </si>
+  <si>
+    <t>10 mg/ml</t>
   </si>
   <si>
     <t>Napa Extra</t>
@@ -1165,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1464,25 +1467,22 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
         <v>69</v>
       </c>
-      <c r="B12" t="s">
-        <v>70</v>
-      </c>
       <c r="C12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="E12" t="s">
         <v>49</v>
       </c>
       <c r="F12">
-        <v>150</v>
+        <v>1000</v>
       </c>
       <c r="G12" s="2">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="H12" t="s">
         <v>50</v>
@@ -1490,25 +1490,25 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E13" t="s">
         <v>49</v>
       </c>
       <c r="F13">
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="G13" s="2">
-        <v>3.5</v>
+        <v>1.4</v>
       </c>
       <c r="H13" t="s">
         <v>50</v>
@@ -1516,27 +1516,53 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14">
+        <v>99</v>
+      </c>
+      <c r="G14" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="H14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="9">
         <v>8</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G15" s="2">
         <v>2.2</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H15" s="9" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>